<commit_message>
feat: initial work on team projection engine
</commit_message>
<xml_diff>
--- a/seasons/2026/output/2026_fantasy_draft_cheat_sheet.xlsx
+++ b/seasons/2026/output/2026_fantasy_draft_cheat_sheet.xlsx
@@ -71,7 +71,7 @@
     <t>2/5</t>
   </si>
   <si>
-    <t>* My Guy</t>
+    <t>My Guy</t>
   </si>
   <si>
     <t>OK near ADP</t>
@@ -191,7 +191,7 @@
     <t>3/5</t>
   </si>
   <si>
-    <t>? Watchlist</t>
+    <t>Watchlist</t>
   </si>
   <si>
     <t>Monitor news</t>
@@ -278,7 +278,7 @@
     <t>4/4</t>
   </si>
   <si>
-    <t>! Value Only</t>
+    <t>Value Only</t>
   </si>
   <si>
     <t>Need discount</t>
@@ -1547,7 +1547,7 @@
     <t>DND</t>
   </si>
   <si>
-    <t>X Do Not Draft</t>
+    <t>Do Not Draft</t>
   </si>
   <si>
     <t>Avoid at normal ADP/cost; only consider after a major fall.</t>

</xml_diff>